<commit_message>
fixed various bugs, added validations on post, added tests
</commit_message>
<xml_diff>
--- a/spec/fixtures/batch_submission_manifest_test.xlsx
+++ b/spec/fixtures/batch_submission_manifest_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FBB4B42-FEA6-2F4E-A96F-89A508CEFC4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D00219F-5B23-5F44-BC12-95CEE2F1B68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="32000" windowHeight="16280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="276">
   <si>
     <t>Field Section</t>
   </si>
@@ -902,6 +902,24 @@
   </si>
   <si>
     <t>not valid</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>not_exist.jpg</t>
+  </si>
+  <si>
+    <t>parent_file_not_found.zip</t>
+  </si>
+  <si>
+    <t>not_found</t>
+  </si>
+  <si>
+    <t>not_both</t>
+  </si>
+  <si>
+    <t>ce447a9f-1500-43d6-83c2-59de00c6ca9c</t>
   </si>
 </sst>
 </file>
@@ -951,7 +969,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1014,12 +1032,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9D2E9"/>
-        <bgColor rgb="FFD9D2E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFEAD1DC"/>
         <bgColor rgb="FFEAD1DC"/>
       </patternFill>
@@ -1043,7 +1055,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -1095,12 +1107,11 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2781,17 +2792,39 @@
       <c r="C8" s="30" t="s">
         <v>249</v>
       </c>
-      <c r="D8" s="31"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
-      <c r="K8" s="30"/>
-      <c r="L8" s="30"/>
-      <c r="M8" s="30"/>
-      <c r="N8" s="30"/>
+      <c r="D8" t="s">
+        <v>271</v>
+      </c>
+      <c r="E8" s="30" t="s">
+        <v>270</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>250</v>
+      </c>
+      <c r="G8" t="s">
+        <v>274</v>
+      </c>
+      <c r="H8" t="s">
+        <v>274</v>
+      </c>
+      <c r="I8" s="30" t="s">
+        <v>273</v>
+      </c>
+      <c r="J8" s="30" t="s">
+        <v>273</v>
+      </c>
+      <c r="K8" s="30" t="s">
+        <v>273</v>
+      </c>
+      <c r="L8" s="30" t="s">
+        <v>273</v>
+      </c>
+      <c r="M8" s="30" t="s">
+        <v>273</v>
+      </c>
+      <c r="N8" s="30" t="s">
+        <v>273</v>
+      </c>
       <c r="O8" s="30" t="s">
         <v>251</v>
       </c>
@@ -2804,24 +2837,22 @@
       <c r="R8" s="30" t="s">
         <v>254</v>
       </c>
-      <c r="S8" s="32"/>
-      <c r="T8" s="32"/>
-      <c r="U8" s="33"/>
-      <c r="V8" s="33"/>
+      <c r="S8" s="31"/>
+      <c r="T8" s="31"/>
+      <c r="U8" s="32"/>
+      <c r="V8" s="32"/>
       <c r="W8" s="30" t="s">
         <v>269</v>
       </c>
-      <c r="X8" s="33"/>
-      <c r="Y8" s="32">
+      <c r="X8" s="32"/>
+      <c r="Y8" s="31">
         <v>2.169024E-2</v>
       </c>
-      <c r="Z8" s="32">
-        <v>2.169024E-2</v>
-      </c>
-      <c r="AA8" s="32">
-        <v>2.169024E-2</v>
-      </c>
-      <c r="AB8" s="32"/>
+      <c r="Z8" s="31"/>
+      <c r="AA8" s="31" t="s">
+        <v>269</v>
+      </c>
+      <c r="AB8" s="31"/>
       <c r="AC8" s="30" t="s">
         <v>269</v>
       </c>
@@ -2859,8 +2890,8 @@
       <c r="AW8" s="30" t="s">
         <v>257</v>
       </c>
-      <c r="AX8" s="32"/>
-      <c r="AY8" s="32"/>
+      <c r="AX8" s="31"/>
+      <c r="AY8" s="31"/>
       <c r="AZ8" s="30" t="s">
         <v>269</v>
       </c>
@@ -2876,24 +2907,24 @@
       <c r="BD8" s="30" t="s">
         <v>269</v>
       </c>
-      <c r="BE8" s="34"/>
-      <c r="BF8" s="32">
+      <c r="BE8" s="33"/>
+      <c r="BF8" s="31">
         <v>3</v>
       </c>
       <c r="BG8" s="30" t="s">
         <v>269</v>
       </c>
-      <c r="BH8" s="32">
+      <c r="BH8" s="31">
         <v>70</v>
       </c>
-      <c r="BI8" s="32">
+      <c r="BI8" s="31">
         <v>1.4E-2</v>
       </c>
-      <c r="BJ8" s="32">
+      <c r="BJ8" s="31">
         <v>200</v>
       </c>
       <c r="BK8" s="30"/>
-      <c r="BL8" s="34"/>
+      <c r="BL8" s="33"/>
       <c r="BM8" s="30" t="s">
         <v>269</v>
       </c>
@@ -2903,20 +2934,20 @@
       <c r="BO8" s="30" t="s">
         <v>269</v>
       </c>
-      <c r="BP8" s="34"/>
+      <c r="BP8" s="33"/>
       <c r="BQ8" s="30" t="s">
         <v>269</v>
       </c>
-      <c r="BR8" s="34"/>
+      <c r="BR8" s="33"/>
       <c r="BS8" s="30" t="s">
         <v>269</v>
       </c>
-      <c r="BT8" s="34"/>
-      <c r="BU8" s="34"/>
-      <c r="BV8" s="34"/>
-      <c r="BW8" s="34"/>
-      <c r="BX8" s="34"/>
-      <c r="BY8" s="34"/>
+      <c r="BT8" s="33"/>
+      <c r="BU8" s="33"/>
+      <c r="BV8" s="33"/>
+      <c r="BW8" s="33"/>
+      <c r="BX8" s="33"/>
+      <c r="BY8" s="33"/>
       <c r="BZ8" s="30" t="s">
         <v>269</v>
       </c>
@@ -2924,8 +2955,8 @@
         <v>269</v>
       </c>
       <c r="CB8" s="30"/>
-      <c r="CC8" s="34"/>
-      <c r="CD8" s="34"/>
+      <c r="CC8" s="33"/>
+      <c r="CD8" s="33"/>
       <c r="CE8" s="30" t="s">
         <v>269</v>
       </c>
@@ -2941,13 +2972,13 @@
       <c r="C9" s="30" t="s">
         <v>259</v>
       </c>
-      <c r="D9" s="35"/>
-      <c r="E9" s="30"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="30" t="s">
+        <v>269</v>
+      </c>
       <c r="F9" s="30" t="s">
-        <v>250</v>
-      </c>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
+        <v>268</v>
+      </c>
       <c r="I9" s="30"/>
       <c r="J9" s="30"/>
       <c r="K9" s="30"/>
@@ -2966,27 +2997,27 @@
       <c r="R9" s="30" t="s">
         <v>254</v>
       </c>
-      <c r="S9" s="32"/>
-      <c r="T9" s="32"/>
-      <c r="U9" s="35"/>
-      <c r="V9" s="35"/>
-      <c r="W9" s="35"/>
-      <c r="X9" s="35"/>
-      <c r="Y9" s="32">
+      <c r="S9" s="31"/>
+      <c r="T9" s="31"/>
+      <c r="U9" s="34"/>
+      <c r="V9" s="34"/>
+      <c r="W9" s="34"/>
+      <c r="X9" s="34"/>
+      <c r="Y9" s="31">
         <v>2.725352E-2</v>
       </c>
-      <c r="Z9" s="32">
+      <c r="Z9" s="31">
         <v>2.725352E-2</v>
       </c>
-      <c r="AA9" s="32">
+      <c r="AA9" s="31">
         <v>2.725352E-2</v>
       </c>
-      <c r="AB9" s="32"/>
-      <c r="AC9" s="32"/>
+      <c r="AB9" s="31"/>
+      <c r="AC9" s="31"/>
       <c r="AD9" s="30" t="s">
         <v>255</v>
       </c>
-      <c r="AE9" s="32"/>
+      <c r="AE9" s="31"/>
       <c r="AF9" s="30"/>
       <c r="AG9" s="30"/>
       <c r="AH9" s="30"/>
@@ -3009,9 +3040,9 @@
       <c r="AW9" s="30" t="s">
         <v>257</v>
       </c>
-      <c r="AX9" s="32"/>
-      <c r="AY9" s="32"/>
-      <c r="AZ9" s="32">
+      <c r="AX9" s="31"/>
+      <c r="AY9" s="31"/>
+      <c r="AZ9" s="31">
         <v>0.200098</v>
       </c>
       <c r="BA9" s="30" t="s">
@@ -3023,44 +3054,44 @@
       <c r="BC9" s="30" t="s">
         <v>256</v>
       </c>
-      <c r="BD9" s="35"/>
-      <c r="BE9" s="35"/>
-      <c r="BF9" s="32">
+      <c r="BD9" s="34"/>
+      <c r="BE9" s="34"/>
+      <c r="BF9" s="31">
         <v>3</v>
       </c>
-      <c r="BG9" s="32">
+      <c r="BG9" s="31">
         <v>1680</v>
       </c>
-      <c r="BH9" s="32">
+      <c r="BH9" s="31">
         <v>70</v>
       </c>
-      <c r="BI9" s="32">
+      <c r="BI9" s="31">
         <v>1.54E-2</v>
       </c>
-      <c r="BJ9" s="32">
+      <c r="BJ9" s="31">
         <v>220</v>
       </c>
       <c r="BK9" s="30"/>
-      <c r="BL9" s="35"/>
-      <c r="BM9" s="35"/>
-      <c r="BN9" s="35"/>
-      <c r="BO9" s="35"/>
-      <c r="BP9" s="35"/>
-      <c r="BQ9" s="35"/>
-      <c r="BR9" s="35"/>
-      <c r="BS9" s="35"/>
-      <c r="BT9" s="35"/>
-      <c r="BU9" s="35"/>
-      <c r="BV9" s="35"/>
-      <c r="BW9" s="35"/>
-      <c r="BX9" s="35"/>
-      <c r="BY9" s="35"/>
+      <c r="BL9" s="34"/>
+      <c r="BM9" s="34"/>
+      <c r="BN9" s="34"/>
+      <c r="BO9" s="34"/>
+      <c r="BP9" s="34"/>
+      <c r="BQ9" s="34"/>
+      <c r="BR9" s="34"/>
+      <c r="BS9" s="34"/>
+      <c r="BT9" s="34"/>
+      <c r="BU9" s="34"/>
+      <c r="BV9" s="34"/>
+      <c r="BW9" s="34"/>
+      <c r="BX9" s="34"/>
+      <c r="BY9" s="34"/>
       <c r="BZ9" s="30"/>
       <c r="CA9" s="30"/>
       <c r="CB9" s="30"/>
-      <c r="CC9" s="35"/>
-      <c r="CD9" s="35"/>
-      <c r="CE9" s="35"/>
+      <c r="CC9" s="34"/>
+      <c r="CD9" s="34"/>
+      <c r="CE9" s="34"/>
       <c r="CF9" s="30" t="s">
         <v>257</v>
       </c>
@@ -3073,15 +3104,18 @@
       <c r="C10" s="30" t="s">
         <v>260</v>
       </c>
-      <c r="D10" s="35"/>
+      <c r="D10" s="34"/>
       <c r="E10" s="30"/>
       <c r="F10" s="30" t="s">
         <v>265</v>
       </c>
-      <c r="G10" s="35"/>
-      <c r="H10" s="35"/>
+      <c r="H10" t="s">
+        <v>273</v>
+      </c>
       <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="30" t="s">
+        <v>275</v>
+      </c>
       <c r="K10" s="30"/>
       <c r="L10" s="30"/>
       <c r="M10" s="30"/>
@@ -3098,27 +3132,27 @@
       <c r="R10" s="30" t="s">
         <v>254</v>
       </c>
-      <c r="S10" s="32"/>
-      <c r="T10" s="32"/>
-      <c r="U10" s="35"/>
-      <c r="V10" s="35"/>
-      <c r="W10" s="35"/>
-      <c r="X10" s="35"/>
-      <c r="Y10" s="32">
+      <c r="S10" s="31"/>
+      <c r="T10" s="31"/>
+      <c r="U10" s="34"/>
+      <c r="V10" s="34"/>
+      <c r="W10" s="34"/>
+      <c r="X10" s="34"/>
+      <c r="Y10" s="31">
         <v>1.5365230000000001E-2</v>
       </c>
-      <c r="Z10" s="32">
+      <c r="Z10" s="31">
         <v>1.5365230000000001E-2</v>
       </c>
-      <c r="AA10" s="32">
+      <c r="AA10" s="31">
         <v>1.5365230000000001E-2</v>
       </c>
-      <c r="AB10" s="32"/>
-      <c r="AC10" s="32"/>
+      <c r="AB10" s="31"/>
+      <c r="AC10" s="31"/>
       <c r="AD10" s="30" t="s">
         <v>255</v>
       </c>
-      <c r="AE10" s="32"/>
+      <c r="AE10" s="31"/>
       <c r="AF10" s="30"/>
       <c r="AG10" s="30"/>
       <c r="AH10" s="30"/>
@@ -3141,9 +3175,9 @@
       <c r="AW10" s="30" t="s">
         <v>257</v>
       </c>
-      <c r="AX10" s="32"/>
-      <c r="AY10" s="32"/>
-      <c r="AZ10" s="32">
+      <c r="AX10" s="31"/>
+      <c r="AY10" s="31"/>
+      <c r="AZ10" s="31">
         <v>0.200098</v>
       </c>
       <c r="BA10" s="30" t="s">
@@ -3155,44 +3189,44 @@
       <c r="BC10" s="30" t="s">
         <v>256</v>
       </c>
-      <c r="BD10" s="35"/>
-      <c r="BE10" s="35"/>
-      <c r="BF10" s="32">
+      <c r="BD10" s="34"/>
+      <c r="BE10" s="34"/>
+      <c r="BF10" s="31">
         <v>3</v>
       </c>
-      <c r="BG10" s="32">
+      <c r="BG10" s="31">
         <v>1680</v>
       </c>
-      <c r="BH10" s="32">
+      <c r="BH10" s="31">
         <v>70</v>
       </c>
-      <c r="BI10" s="32">
+      <c r="BI10" s="31">
         <v>1.54E-2</v>
       </c>
-      <c r="BJ10" s="32">
+      <c r="BJ10" s="31">
         <v>220</v>
       </c>
       <c r="BK10" s="30"/>
-      <c r="BL10" s="35"/>
-      <c r="BM10" s="35"/>
-      <c r="BN10" s="35"/>
-      <c r="BO10" s="35"/>
-      <c r="BP10" s="35"/>
-      <c r="BQ10" s="35"/>
-      <c r="BR10" s="35"/>
-      <c r="BS10" s="35"/>
-      <c r="BT10" s="35"/>
-      <c r="BU10" s="35"/>
-      <c r="BV10" s="35"/>
-      <c r="BW10" s="35"/>
-      <c r="BX10" s="35"/>
-      <c r="BY10" s="35"/>
+      <c r="BL10" s="34"/>
+      <c r="BM10" s="34"/>
+      <c r="BN10" s="34"/>
+      <c r="BO10" s="34"/>
+      <c r="BP10" s="34"/>
+      <c r="BQ10" s="34"/>
+      <c r="BR10" s="34"/>
+      <c r="BS10" s="34"/>
+      <c r="BT10" s="34"/>
+      <c r="BU10" s="34"/>
+      <c r="BV10" s="34"/>
+      <c r="BW10" s="34"/>
+      <c r="BX10" s="34"/>
+      <c r="BY10" s="34"/>
       <c r="BZ10" s="30"/>
       <c r="CA10" s="30"/>
       <c r="CB10" s="30"/>
-      <c r="CC10" s="35"/>
-      <c r="CD10" s="35"/>
-      <c r="CE10" s="35"/>
+      <c r="CC10" s="34"/>
+      <c r="CD10" s="34"/>
+      <c r="CE10" s="34"/>
       <c r="CF10" s="30" t="s">
         <v>257</v>
       </c>
@@ -3204,13 +3238,17 @@
       <c r="C11" s="30" t="s">
         <v>261</v>
       </c>
-      <c r="D11" s="35"/>
-      <c r="E11" s="30"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="30" t="s">
+        <v>270</v>
+      </c>
       <c r="F11" s="30" t="s">
         <v>266</v>
       </c>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
+      <c r="G11" t="s">
+        <v>272</v>
+      </c>
+      <c r="H11" s="34"/>
       <c r="I11" s="30"/>
       <c r="J11" s="30"/>
       <c r="K11" s="30"/>
@@ -3229,27 +3267,27 @@
       <c r="R11" s="30" t="s">
         <v>254</v>
       </c>
-      <c r="S11" s="32"/>
-      <c r="T11" s="32"/>
-      <c r="U11" s="35"/>
-      <c r="V11" s="35"/>
-      <c r="W11" s="35"/>
-      <c r="X11" s="35"/>
-      <c r="Y11" s="32">
+      <c r="S11" s="31"/>
+      <c r="T11" s="31"/>
+      <c r="U11" s="34"/>
+      <c r="V11" s="34"/>
+      <c r="W11" s="34"/>
+      <c r="X11" s="34"/>
+      <c r="Y11" s="31">
         <v>4.8993170000000003E-2</v>
       </c>
-      <c r="Z11" s="32">
+      <c r="Z11" s="31">
         <v>4.8993170000000003E-2</v>
       </c>
-      <c r="AA11" s="32">
+      <c r="AA11" s="31">
         <v>4.8993170000000003E-2</v>
       </c>
-      <c r="AB11" s="32"/>
-      <c r="AC11" s="32"/>
+      <c r="AB11" s="31"/>
+      <c r="AC11" s="31"/>
       <c r="AD11" s="30" t="s">
         <v>255</v>
       </c>
-      <c r="AE11" s="32"/>
+      <c r="AE11" s="31"/>
       <c r="AF11" s="30"/>
       <c r="AG11" s="30"/>
       <c r="AH11" s="30"/>
@@ -3272,9 +3310,9 @@
       <c r="AW11" s="30" t="s">
         <v>257</v>
       </c>
-      <c r="AX11" s="32"/>
-      <c r="AY11" s="32"/>
-      <c r="AZ11" s="32">
+      <c r="AX11" s="31"/>
+      <c r="AY11" s="31"/>
+      <c r="AZ11" s="31">
         <v>0.200098</v>
       </c>
       <c r="BA11" s="30" t="s">
@@ -3286,44 +3324,44 @@
       <c r="BC11" s="30" t="s">
         <v>256</v>
       </c>
-      <c r="BD11" s="35"/>
-      <c r="BE11" s="35"/>
-      <c r="BF11" s="32">
+      <c r="BD11" s="34"/>
+      <c r="BE11" s="34"/>
+      <c r="BF11" s="31">
         <v>3</v>
       </c>
-      <c r="BG11" s="32">
+      <c r="BG11" s="31">
         <v>600</v>
       </c>
-      <c r="BH11" s="32">
+      <c r="BH11" s="31">
         <v>70</v>
       </c>
-      <c r="BI11" s="32">
+      <c r="BI11" s="31">
         <v>1.54E-2</v>
       </c>
-      <c r="BJ11" s="32">
+      <c r="BJ11" s="31">
         <v>220</v>
       </c>
       <c r="BK11" s="30"/>
-      <c r="BL11" s="35"/>
-      <c r="BM11" s="35"/>
-      <c r="BN11" s="35"/>
-      <c r="BO11" s="35"/>
-      <c r="BP11" s="35"/>
-      <c r="BQ11" s="35"/>
-      <c r="BR11" s="35"/>
-      <c r="BS11" s="35"/>
-      <c r="BT11" s="35"/>
-      <c r="BU11" s="35"/>
-      <c r="BV11" s="35"/>
-      <c r="BW11" s="35"/>
-      <c r="BX11" s="35"/>
-      <c r="BY11" s="35"/>
+      <c r="BL11" s="34"/>
+      <c r="BM11" s="34"/>
+      <c r="BN11" s="34"/>
+      <c r="BO11" s="34"/>
+      <c r="BP11" s="34"/>
+      <c r="BQ11" s="34"/>
+      <c r="BR11" s="34"/>
+      <c r="BS11" s="34"/>
+      <c r="BT11" s="34"/>
+      <c r="BU11" s="34"/>
+      <c r="BV11" s="34"/>
+      <c r="BW11" s="34"/>
+      <c r="BX11" s="34"/>
+      <c r="BY11" s="34"/>
       <c r="BZ11" s="30"/>
       <c r="CA11" s="30"/>
       <c r="CB11" s="30"/>
-      <c r="CC11" s="35"/>
-      <c r="CD11" s="35"/>
-      <c r="CE11" s="35"/>
+      <c r="CC11" s="34"/>
+      <c r="CD11" s="34"/>
+      <c r="CE11" s="34"/>
       <c r="CF11" s="30" t="s">
         <v>257</v>
       </c>
@@ -3335,13 +3373,17 @@
       <c r="C12" s="30" t="s">
         <v>263</v>
       </c>
-      <c r="D12" s="35"/>
-      <c r="E12" s="30"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="30" t="s">
+        <v>270</v>
+      </c>
       <c r="F12" s="30" t="s">
         <v>267</v>
       </c>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
+      <c r="G12" s="30" t="s">
+        <v>263</v>
+      </c>
+      <c r="H12" s="34"/>
       <c r="I12" s="30"/>
       <c r="J12" s="30"/>
       <c r="K12" s="30"/>
@@ -3360,27 +3402,27 @@
       <c r="R12" s="30" t="s">
         <v>254</v>
       </c>
-      <c r="S12" s="32"/>
-      <c r="T12" s="32"/>
-      <c r="U12" s="35"/>
-      <c r="V12" s="35"/>
-      <c r="W12" s="35"/>
-      <c r="X12" s="35"/>
-      <c r="Y12" s="32">
+      <c r="S12" s="31"/>
+      <c r="T12" s="31"/>
+      <c r="U12" s="34"/>
+      <c r="V12" s="34"/>
+      <c r="W12" s="34"/>
+      <c r="X12" s="34"/>
+      <c r="Y12" s="31">
         <v>1.4276580000000001E-2</v>
       </c>
-      <c r="Z12" s="32">
+      <c r="Z12" s="31">
         <v>1.4276580000000001E-2</v>
       </c>
-      <c r="AA12" s="32">
+      <c r="AA12" s="31">
         <v>1.4276580000000001E-2</v>
       </c>
-      <c r="AB12" s="32"/>
-      <c r="AC12" s="32"/>
+      <c r="AB12" s="31"/>
+      <c r="AC12" s="31"/>
       <c r="AD12" s="30" t="s">
         <v>255</v>
       </c>
-      <c r="AE12" s="32"/>
+      <c r="AE12" s="31"/>
       <c r="AF12" s="30"/>
       <c r="AG12" s="30"/>
       <c r="AH12" s="30"/>
@@ -3403,9 +3445,9 @@
       <c r="AW12" s="30" t="s">
         <v>257</v>
       </c>
-      <c r="AX12" s="32"/>
-      <c r="AY12" s="32"/>
-      <c r="AZ12" s="32">
+      <c r="AX12" s="31"/>
+      <c r="AY12" s="31"/>
+      <c r="AZ12" s="31">
         <v>0.200098</v>
       </c>
       <c r="BA12" s="30" t="s">
@@ -3417,44 +3459,44 @@
       <c r="BC12" s="30" t="s">
         <v>256</v>
       </c>
-      <c r="BD12" s="35"/>
-      <c r="BE12" s="35"/>
-      <c r="BF12" s="32">
+      <c r="BD12" s="34"/>
+      <c r="BE12" s="34"/>
+      <c r="BF12" s="31">
         <v>3</v>
       </c>
-      <c r="BG12" s="32">
+      <c r="BG12" s="31">
         <v>1440</v>
       </c>
-      <c r="BH12" s="32">
+      <c r="BH12" s="31">
         <v>70</v>
       </c>
-      <c r="BI12" s="32">
+      <c r="BI12" s="31">
         <v>1.4E-2</v>
       </c>
-      <c r="BJ12" s="32">
+      <c r="BJ12" s="31">
         <v>200</v>
       </c>
       <c r="BK12" s="30"/>
-      <c r="BL12" s="35"/>
-      <c r="BM12" s="35"/>
-      <c r="BN12" s="35"/>
-      <c r="BO12" s="35"/>
-      <c r="BP12" s="35"/>
-      <c r="BQ12" s="35"/>
-      <c r="BR12" s="35"/>
-      <c r="BS12" s="35"/>
-      <c r="BT12" s="35"/>
-      <c r="BU12" s="35"/>
-      <c r="BV12" s="35"/>
-      <c r="BW12" s="35"/>
-      <c r="BX12" s="35"/>
-      <c r="BY12" s="35"/>
+      <c r="BL12" s="34"/>
+      <c r="BM12" s="34"/>
+      <c r="BN12" s="34"/>
+      <c r="BO12" s="34"/>
+      <c r="BP12" s="34"/>
+      <c r="BQ12" s="34"/>
+      <c r="BR12" s="34"/>
+      <c r="BS12" s="34"/>
+      <c r="BT12" s="34"/>
+      <c r="BU12" s="34"/>
+      <c r="BV12" s="34"/>
+      <c r="BW12" s="34"/>
+      <c r="BX12" s="34"/>
+      <c r="BY12" s="34"/>
       <c r="BZ12" s="30"/>
       <c r="CA12" s="30"/>
       <c r="CB12" s="30"/>
-      <c r="CC12" s="35"/>
-      <c r="CD12" s="35"/>
-      <c r="CE12" s="35"/>
+      <c r="CC12" s="34"/>
+      <c r="CD12" s="34"/>
+      <c r="CE12" s="34"/>
       <c r="CF12" s="30" t="s">
         <v>257</v>
       </c>
@@ -3466,13 +3508,13 @@
       <c r="C13" s="30" t="s">
         <v>264</v>
       </c>
-      <c r="D13" s="35"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30" t="s">
-        <v>268</v>
-      </c>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="30" t="s">
+        <v>270</v>
+      </c>
+      <c r="F13" s="30"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
       <c r="I13" s="30"/>
       <c r="J13" s="30"/>
       <c r="K13" s="30"/>
@@ -3491,27 +3533,27 @@
       <c r="R13" s="30" t="s">
         <v>254</v>
       </c>
-      <c r="S13" s="32"/>
-      <c r="T13" s="32"/>
-      <c r="U13" s="35"/>
-      <c r="V13" s="35"/>
-      <c r="W13" s="35"/>
-      <c r="X13" s="35"/>
-      <c r="Y13" s="32">
+      <c r="S13" s="31"/>
+      <c r="T13" s="31"/>
+      <c r="U13" s="34"/>
+      <c r="V13" s="34"/>
+      <c r="W13" s="34"/>
+      <c r="X13" s="34"/>
+      <c r="Y13" s="31">
         <v>2.725352E-2</v>
       </c>
-      <c r="Z13" s="32">
+      <c r="Z13" s="31">
         <v>2.725352E-2</v>
       </c>
-      <c r="AA13" s="32">
+      <c r="AA13" s="31">
         <v>2.725352E-2</v>
       </c>
-      <c r="AB13" s="32"/>
-      <c r="AC13" s="32"/>
+      <c r="AB13" s="31"/>
+      <c r="AC13" s="31"/>
       <c r="AD13" s="30" t="s">
         <v>255</v>
       </c>
-      <c r="AE13" s="32"/>
+      <c r="AE13" s="31"/>
       <c r="AF13" s="30"/>
       <c r="AG13" s="30"/>
       <c r="AH13" s="30"/>
@@ -3534,9 +3576,9 @@
       <c r="AW13" s="30" t="s">
         <v>257</v>
       </c>
-      <c r="AX13" s="32"/>
-      <c r="AY13" s="32"/>
-      <c r="AZ13" s="32">
+      <c r="AX13" s="31"/>
+      <c r="AY13" s="31"/>
+      <c r="AZ13" s="31">
         <v>0.200098</v>
       </c>
       <c r="BA13" s="30" t="s">
@@ -3548,44 +3590,44 @@
       <c r="BC13" s="30" t="s">
         <v>256</v>
       </c>
-      <c r="BD13" s="35"/>
-      <c r="BE13" s="35"/>
-      <c r="BF13" s="32">
+      <c r="BD13" s="34"/>
+      <c r="BE13" s="34"/>
+      <c r="BF13" s="31">
         <v>3</v>
       </c>
-      <c r="BG13" s="32">
+      <c r="BG13" s="31">
         <v>1680</v>
       </c>
-      <c r="BH13" s="32">
+      <c r="BH13" s="31">
         <v>70</v>
       </c>
-      <c r="BI13" s="32">
+      <c r="BI13" s="31">
         <v>1.54E-2</v>
       </c>
-      <c r="BJ13" s="32">
+      <c r="BJ13" s="31">
         <v>220</v>
       </c>
       <c r="BK13" s="30"/>
-      <c r="BL13" s="35"/>
-      <c r="BM13" s="35"/>
-      <c r="BN13" s="35"/>
-      <c r="BO13" s="35"/>
-      <c r="BP13" s="35"/>
-      <c r="BQ13" s="35"/>
-      <c r="BR13" s="35"/>
-      <c r="BS13" s="35"/>
-      <c r="BT13" s="35"/>
-      <c r="BU13" s="35"/>
-      <c r="BV13" s="35"/>
-      <c r="BW13" s="35"/>
-      <c r="BX13" s="35"/>
-      <c r="BY13" s="35"/>
+      <c r="BL13" s="34"/>
+      <c r="BM13" s="34"/>
+      <c r="BN13" s="34"/>
+      <c r="BO13" s="34"/>
+      <c r="BP13" s="34"/>
+      <c r="BQ13" s="34"/>
+      <c r="BR13" s="34"/>
+      <c r="BS13" s="34"/>
+      <c r="BT13" s="34"/>
+      <c r="BU13" s="34"/>
+      <c r="BV13" s="34"/>
+      <c r="BW13" s="34"/>
+      <c r="BX13" s="34"/>
+      <c r="BY13" s="34"/>
       <c r="BZ13" s="30"/>
       <c r="CA13" s="30"/>
       <c r="CB13" s="30"/>
-      <c r="CC13" s="35"/>
-      <c r="CD13" s="35"/>
-      <c r="CE13" s="35"/>
+      <c r="CC13" s="34"/>
+      <c r="CD13" s="34"/>
+      <c r="CE13" s="34"/>
       <c r="CF13" s="30" t="s">
         <v>257</v>
       </c>

</xml_diff>